<commit_message>
v5: fix reference sheet banners — data shared by client, not yet in CRM
The previous banners said 'already imported into CRM' which was wrong.
Nothing is in CRM yet — Alison has shared 3 modules of data
(Client Accounts, Clients, Investigators) and still needs to fill
Instructions + Premises in this template before we can run the
full 6-module import.

New banner text:
  Client Accounts — law firms you've already shared with us. Add any new firms in the empty rows below.
  Clients — lawyers you've already shared with us. Add any new contacts in the empty rows below.
  Investigators — investigators you've already shared with us. Add any new investigators in the empty rows below.

Project #4593 — A2Z Cloud
</commit_message>
<xml_diff>
--- a/ID Inquiries/Migration/4593_ID_Inquiries_Migration_Intake_v5.xlsx
+++ b/ID Inquiries/Migration/4593_ID_Inquiries_Migration_Intake_v5.xlsx
@@ -14053,7 +14053,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Client Accounts — law firms already imported into CRM. Edit only if details are outdated. Add new firms in the empty rows below.</t>
+          <t>Client Accounts — law firms you've already shared with us. Add any new firms in the empty rows below.</t>
         </is>
       </c>
     </row>
@@ -15421,7 +15421,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Clients — individual lawyers already imported into CRM. Edit only if details are outdated. Add new clients in the empty rows below.</t>
+          <t>Clients — lawyers you've already shared with us. Add any new contacts in the empty rows below.</t>
         </is>
       </c>
     </row>
@@ -16048,7 +16048,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Investigators — field investigators already imported into CRM. Edit only if details are outdated. Add new investigators in the empty rows below.</t>
+          <t>Investigators — investigators you've already shared with us. Add any new investigators in the empty rows below.</t>
         </is>
       </c>
     </row>

</xml_diff>